<commit_message>
Update camera_events.xlsx (Samsara weekly refresh 2026-08-09)
</commit_message>
<xml_diff>
--- a/camera_events.xlsx
+++ b/camera_events.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Shared drives\Synergy Safety Group\DEN\Dashboard\Weekly Dashboards\Mott-s-Wrecker-Service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D9AC9E2-5C37-4103-BEF1-694CCA01BC5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{498B8D85-4B41-4B6C-B9E6-7FC3132D6164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2895" yWindow="2895" windowWidth="43200" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DRIVE-ALERTS" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8019" uniqueCount="3712">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8187" uniqueCount="3799">
   <si>
     <t>DRIVE ALERTS</t>
   </si>
@@ -9247,21 +9247,21 @@
     <t>06/19/26 16:32 EDT</t>
   </si>
   <si>
+    <t>1.9mi S of Kirby TX</t>
+  </si>
+  <si>
+    <t>29.433548, -98.390060</t>
+  </si>
+  <si>
+    <t>06/21/26 21:00 EDT</t>
+  </si>
+  <si>
     <t>COLLISION-WARNING</t>
   </si>
   <si>
-    <t>1.9mi S of Kirby TX</t>
-  </si>
-  <si>
-    <t>29.433548, -98.390060</t>
-  </si>
-  <si>
     <t>06/22/26 13:05 EDT</t>
   </si>
   <si>
-    <t>06/21/26 21:00 EDT</t>
-  </si>
-  <si>
     <t>06/19/26 16:36 EDT</t>
   </si>
   <si>
@@ -10972,7 +10972,7 @@
     <t>29.636524, -97.729690</t>
   </si>
   <si>
-    <t>07/28/26 20:56 EDT</t>
+    <t>08/04/26 20:55 EDT</t>
   </si>
   <si>
     <t>07/28/26 13:59 EDT</t>
@@ -10999,9 +10999,6 @@
     <t>29.582280, -97.999500</t>
   </si>
   <si>
-    <t>07/30/26 08:15 EDT</t>
-  </si>
-  <si>
     <t>07/29/26 14:48 EDT</t>
   </si>
   <si>
@@ -11110,7 +11107,10 @@
     <t>29.215775, -98.802870</t>
   </si>
   <si>
-    <t>08/03/26 07:13 EDT</t>
+    <t>08/03/26 17:55 EDT</t>
+  </si>
+  <si>
+    <t>08/03/26 18:38 EDT</t>
   </si>
   <si>
     <t>08/02/26 22:03 EDT</t>
@@ -11156,6 +11156,267 @@
   </si>
   <si>
     <t>29.132158, -98.893130</t>
+  </si>
+  <si>
+    <t>08/03/26 13:03 EDT</t>
+  </si>
+  <si>
+    <t>8.5mi E of Seguin TX</t>
+  </si>
+  <si>
+    <t>29.614721, -97.829750</t>
+  </si>
+  <si>
+    <t>08/03/26 13:59 EDT</t>
+  </si>
+  <si>
+    <t>29.503805, -98.288460</t>
+  </si>
+  <si>
+    <t>08/03/26 18:00 EDT</t>
+  </si>
+  <si>
+    <t>08/03/26 14:59 EDT</t>
+  </si>
+  <si>
+    <t>2.9mi SW of Seguin TX</t>
+  </si>
+  <si>
+    <t>29.571743, -98.010666</t>
+  </si>
+  <si>
+    <t>08/03/26 16:59 EDT</t>
+  </si>
+  <si>
+    <t>29.502413, -98.183330</t>
+  </si>
+  <si>
+    <t>08/04/26 12:27 EDT</t>
+  </si>
+  <si>
+    <t>7.8mi NW of Fredericksburg TX</t>
+  </si>
+  <si>
+    <t>30.364586, -98.939190</t>
+  </si>
+  <si>
+    <t>08/04/26 12:53 EDT</t>
+  </si>
+  <si>
+    <t>31.5mi S of Brady TX</t>
+  </si>
+  <si>
+    <t>30.704916, -99.184570</t>
+  </si>
+  <si>
+    <t>08/04/26 13:59 EDT</t>
+  </si>
+  <si>
+    <t>13mi NW of Fredericksburg TX</t>
+  </si>
+  <si>
+    <t>30.433535, -98.973076</t>
+  </si>
+  <si>
+    <t>08/04/26 15:42 EDT</t>
+  </si>
+  <si>
+    <t>6.6mi S of Timberwood Park TX</t>
+  </si>
+  <si>
+    <t>29.606453, -98.458760</t>
+  </si>
+  <si>
+    <t>08/04/26 15:49 EDT</t>
+  </si>
+  <si>
+    <t>3.5mi W of Selma TX</t>
+  </si>
+  <si>
+    <t>29.602657, -98.368996</t>
+  </si>
+  <si>
+    <t>08/05/26 09:24 EDT</t>
+  </si>
+  <si>
+    <t>15.3mi SE of Cibolo TX</t>
+  </si>
+  <si>
+    <t>29.363966, -98.100950</t>
+  </si>
+  <si>
+    <t>08/06/26 07:52 EDT</t>
+  </si>
+  <si>
+    <t>08/05/26 09:33 EDT</t>
+  </si>
+  <si>
+    <t>4.3mi NW of Seguin TX</t>
+  </si>
+  <si>
+    <t>29.627094, -98.023550</t>
+  </si>
+  <si>
+    <t>08/05/26 10:53 EDT</t>
+  </si>
+  <si>
+    <t>29.492538, -98.121060</t>
+  </si>
+  <si>
+    <t>08/05/26 11:18 EDT</t>
+  </si>
+  <si>
+    <t>08/05/26 13:27 EDT</t>
+  </si>
+  <si>
+    <t>5.2mi N of Cibolo TX</t>
+  </si>
+  <si>
+    <t>29.639088, -98.213610</t>
+  </si>
+  <si>
+    <t>08/05/26 16:59 EDT</t>
+  </si>
+  <si>
+    <t>41.4mi NW of Kerrville TX</t>
+  </si>
+  <si>
+    <t>30.416855, -99.671570</t>
+  </si>
+  <si>
+    <t>08/05/26 20:02 EDT</t>
+  </si>
+  <si>
+    <t>2mi NW of Kirby TX</t>
+  </si>
+  <si>
+    <t>29.486227, -98.402860</t>
+  </si>
+  <si>
+    <t>08/06/26 08:44 EDT</t>
+  </si>
+  <si>
+    <t>8.3mi S of Lackland AFB TX</t>
+  </si>
+  <si>
+    <t>29.272161, -98.574120</t>
+  </si>
+  <si>
+    <t>08/06/26 12:55 EDT</t>
+  </si>
+  <si>
+    <t>7.5mi SE of Lackland AFB TX</t>
+  </si>
+  <si>
+    <t>29.292131, -98.557970</t>
+  </si>
+  <si>
+    <t>08/06/26 14:02 EDT</t>
+  </si>
+  <si>
+    <t>3.5mi NE of New Braunfels TX</t>
+  </si>
+  <si>
+    <t>29.733608, -98.072540</t>
+  </si>
+  <si>
+    <t>08/07/26 07:43 EDT</t>
+  </si>
+  <si>
+    <t>08/06/26 14:10 EDT</t>
+  </si>
+  <si>
+    <t>4mi SW of San Marcos TX</t>
+  </si>
+  <si>
+    <t>29.831070, -97.981720</t>
+  </si>
+  <si>
+    <t>08/07/26 07:46 EDT</t>
+  </si>
+  <si>
+    <t>08/06/26 19:29 EDT</t>
+  </si>
+  <si>
+    <t>3mi E of Cibolo TX</t>
+  </si>
+  <si>
+    <t>29.567762, -98.162280</t>
+  </si>
+  <si>
+    <t>08/06/26 21:15 EDT</t>
+  </si>
+  <si>
+    <t>3.4mi SW of Seguin TX</t>
+  </si>
+  <si>
+    <t>29.569626, -98.018814</t>
+  </si>
+  <si>
+    <t>08/06/26 21:18 EDT</t>
+  </si>
+  <si>
+    <t>6.3mi SW of Seguin TX</t>
+  </si>
+  <si>
+    <t>29.545012, -98.058846</t>
+  </si>
+  <si>
+    <t>08/07/26 08:53 EDT</t>
+  </si>
+  <si>
+    <t>08/07/26 10:22 EDT</t>
+  </si>
+  <si>
+    <t>28mi SE of Floresville TX</t>
+  </si>
+  <si>
+    <t>28.834064, -97.867850</t>
+  </si>
+  <si>
+    <t>08/07/26 15:29 EDT</t>
+  </si>
+  <si>
+    <t>17.1mi S of Pearsall TX</t>
+  </si>
+  <si>
+    <t>28.655476, -99.180374</t>
+  </si>
+  <si>
+    <t>08/07/26 15:59 EDT</t>
+  </si>
+  <si>
+    <t>16.2mi NE of Pearsall TX</t>
+  </si>
+  <si>
+    <t>29.090797, -98.955086</t>
+  </si>
+  <si>
+    <t>08/07/26 17:00 EDT</t>
+  </si>
+  <si>
+    <t>28.790812, -97.773094</t>
+  </si>
+  <si>
+    <t>08/07/26 21:34 EDT</t>
+  </si>
+  <si>
+    <t>08/08/26 10:33 EDT</t>
+  </si>
+  <si>
+    <t>26.4mi N of Beeville TX</t>
+  </si>
+  <si>
+    <t>28.787094, -97.766130</t>
+  </si>
+  <si>
+    <t>08/08/26 11:47 EDT</t>
+  </si>
+  <si>
+    <t>4.5mi NW of Floresville TX</t>
+  </si>
+  <si>
+    <t>29.198547, -98.206930</t>
   </si>
 </sst>
 </file>
@@ -11517,7 +11778,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N1317"/>
+  <dimension ref="A1:N1345"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="14" width="15" customWidth="1"/>
@@ -35270,7 +35531,7 @@
         <v>112</v>
       </c>
       <c r="D742" s="3">
-        <v>5622402770</v>
+        <v>5622271458</v>
       </c>
       <c r="E742" s="3" t="s">
         <v>53</v>
@@ -35300,7 +35561,7 @@
         <v>112</v>
       </c>
       <c r="D743" s="3">
-        <v>5622271458</v>
+        <v>5622402770</v>
       </c>
       <c r="E743" s="3" t="s">
         <v>53</v>
@@ -46728,16 +46989,16 @@
         <v>112</v>
       </c>
       <c r="D1095" s="3">
-        <v>5982274613</v>
+        <v>5982274614</v>
       </c>
       <c r="E1095" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="F1095" s="3" t="s">
         <v>3075</v>
       </c>
-      <c r="F1095" s="3" t="s">
+      <c r="G1095" s="3" t="s">
         <v>3076</v>
-      </c>
-      <c r="G1095" s="3" t="s">
-        <v>3077</v>
       </c>
       <c r="H1095" s="3" t="s">
         <v>110</v>
@@ -46751,7 +47012,7 @@
         <v>39</v>
       </c>
       <c r="M1095" s="3" t="s">
-        <v>3078</v>
+        <v>3077</v>
       </c>
       <c r="N1095" s="3"/>
     </row>
@@ -46764,16 +47025,16 @@
         <v>112</v>
       </c>
       <c r="D1096" s="3">
-        <v>5982274614</v>
+        <v>5982274613</v>
       </c>
       <c r="E1096" s="3" t="s">
-        <v>428</v>
+        <v>3078</v>
       </c>
       <c r="F1096" s="3" t="s">
+        <v>3075</v>
+      </c>
+      <c r="G1096" s="3" t="s">
         <v>3076</v>
-      </c>
-      <c r="G1096" s="3" t="s">
-        <v>3077</v>
       </c>
       <c r="H1096" s="3" t="s">
         <v>110</v>
@@ -49904,7 +50165,7 @@
         <v>71</v>
       </c>
       <c r="F1194" s="3" t="s">
-        <v>3076</v>
+        <v>3075</v>
       </c>
       <c r="G1194" s="3" t="s">
         <v>3351</v>
@@ -53164,7 +53425,7 @@
         <v>3649</v>
       </c>
       <c r="H1295" s="3" t="s">
-        <v>110</v>
+        <v>1678</v>
       </c>
       <c r="I1295" s="3"/>
       <c r="J1295" s="3"/>
@@ -53290,7 +53551,7 @@
         <v>3658</v>
       </c>
       <c r="H1299" s="3" t="s">
-        <v>110</v>
+        <v>1678</v>
       </c>
       <c r="I1299" s="3"/>
       <c r="J1299" s="3"/>
@@ -53301,13 +53562,13 @@
         <v>39</v>
       </c>
       <c r="M1299" s="3" t="s">
-        <v>3659</v>
+        <v>3650</v>
       </c>
       <c r="N1299" s="3"/>
     </row>
     <row r="1300" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1300" s="3" t="s">
-        <v>3660</v>
+        <v>3659</v>
       </c>
       <c r="B1300" s="3"/>
       <c r="C1300" s="3">
@@ -53323,10 +53584,10 @@
         <v>47</v>
       </c>
       <c r="G1300" s="3" t="s">
-        <v>3661</v>
+        <v>3660</v>
       </c>
       <c r="H1300" s="3" t="s">
-        <v>110</v>
+        <v>1678</v>
       </c>
       <c r="I1300" s="3"/>
       <c r="J1300" s="3"/>
@@ -53337,13 +53598,13 @@
         <v>39</v>
       </c>
       <c r="M1300" s="3" t="s">
-        <v>3659</v>
+        <v>3650</v>
       </c>
       <c r="N1300" s="3"/>
     </row>
     <row r="1301" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1301" s="3" t="s">
-        <v>3662</v>
+        <v>3661</v>
       </c>
       <c r="B1301" s="3"/>
       <c r="C1301" s="3">
@@ -53359,7 +53620,7 @@
         <v>869</v>
       </c>
       <c r="G1301" s="3" t="s">
-        <v>3663</v>
+        <v>3662</v>
       </c>
       <c r="H1301" s="3"/>
       <c r="I1301" s="3"/>
@@ -53373,7 +53634,7 @@
     </row>
     <row r="1302" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1302" s="3" t="s">
-        <v>3664</v>
+        <v>3663</v>
       </c>
       <c r="B1302" s="3"/>
       <c r="C1302" s="3">
@@ -53389,7 +53650,7 @@
         <v>230</v>
       </c>
       <c r="G1302" s="3" t="s">
-        <v>3665</v>
+        <v>3664</v>
       </c>
       <c r="H1302" s="3"/>
       <c r="I1302" s="3"/>
@@ -53403,7 +53664,7 @@
     </row>
     <row r="1303" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1303" s="3" t="s">
-        <v>3666</v>
+        <v>3665</v>
       </c>
       <c r="B1303" s="3"/>
       <c r="C1303" s="3">
@@ -53416,10 +53677,10 @@
         <v>80</v>
       </c>
       <c r="F1303" s="3" t="s">
+        <v>3666</v>
+      </c>
+      <c r="G1303" s="3" t="s">
         <v>3667</v>
-      </c>
-      <c r="G1303" s="3" t="s">
-        <v>3668</v>
       </c>
       <c r="H1303" s="3" t="s">
         <v>110</v>
@@ -53433,13 +53694,13 @@
         <v>39</v>
       </c>
       <c r="M1303" s="3" t="s">
-        <v>3669</v>
+        <v>3668</v>
       </c>
       <c r="N1303" s="3"/>
     </row>
     <row r="1304" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1304" s="3" t="s">
-        <v>3670</v>
+        <v>3669</v>
       </c>
       <c r="B1304" s="3"/>
       <c r="C1304" s="3">
@@ -53455,7 +53716,7 @@
         <v>1832</v>
       </c>
       <c r="G1304" s="3" t="s">
-        <v>3671</v>
+        <v>3670</v>
       </c>
       <c r="H1304" s="3"/>
       <c r="I1304" s="3"/>
@@ -53469,7 +53730,7 @@
     </row>
     <row r="1305" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1305" s="3" t="s">
-        <v>3672</v>
+        <v>3671</v>
       </c>
       <c r="B1305" s="3"/>
       <c r="C1305" s="3">
@@ -53485,7 +53746,7 @@
         <v>230</v>
       </c>
       <c r="G1305" s="3" t="s">
-        <v>3673</v>
+        <v>3672</v>
       </c>
       <c r="H1305" s="3" t="s">
         <v>110</v>
@@ -53499,13 +53760,13 @@
         <v>39</v>
       </c>
       <c r="M1305" s="3" t="s">
-        <v>3674</v>
+        <v>3673</v>
       </c>
       <c r="N1305" s="3"/>
     </row>
     <row r="1306" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1306" s="3" t="s">
-        <v>3675</v>
+        <v>3674</v>
       </c>
       <c r="B1306" s="3"/>
       <c r="C1306" s="3">
@@ -53518,10 +53779,10 @@
         <v>53</v>
       </c>
       <c r="F1306" s="3" t="s">
+        <v>3675</v>
+      </c>
+      <c r="G1306" s="3" t="s">
         <v>3676</v>
-      </c>
-      <c r="G1306" s="3" t="s">
-        <v>3677</v>
       </c>
       <c r="H1306" s="3"/>
       <c r="I1306" s="3"/>
@@ -53535,7 +53796,7 @@
     </row>
     <row r="1307" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1307" s="3" t="s">
-        <v>3678</v>
+        <v>3677</v>
       </c>
       <c r="B1307" s="3"/>
       <c r="C1307" s="3">
@@ -53551,7 +53812,7 @@
         <v>990</v>
       </c>
       <c r="G1307" s="3" t="s">
-        <v>3679</v>
+        <v>3678</v>
       </c>
       <c r="H1307" s="3" t="s">
         <v>110</v>
@@ -53565,13 +53826,13 @@
         <v>39</v>
       </c>
       <c r="M1307" s="3" t="s">
-        <v>3680</v>
+        <v>3679</v>
       </c>
       <c r="N1307" s="3"/>
     </row>
     <row r="1308" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1308" s="3" t="s">
-        <v>3678</v>
+        <v>3677</v>
       </c>
       <c r="B1308" s="3"/>
       <c r="C1308" s="3">
@@ -53587,7 +53848,7 @@
         <v>557</v>
       </c>
       <c r="G1308" s="3" t="s">
-        <v>3681</v>
+        <v>3680</v>
       </c>
       <c r="H1308" s="3" t="s">
         <v>110</v>
@@ -53601,13 +53862,13 @@
         <v>39</v>
       </c>
       <c r="M1308" s="3" t="s">
-        <v>3680</v>
+        <v>3679</v>
       </c>
       <c r="N1308" s="3"/>
     </row>
     <row r="1309" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1309" s="3" t="s">
-        <v>3682</v>
+        <v>3681</v>
       </c>
       <c r="B1309" s="3"/>
       <c r="C1309" s="3">
@@ -53623,7 +53884,7 @@
         <v>230</v>
       </c>
       <c r="G1309" s="3" t="s">
-        <v>3683</v>
+        <v>3682</v>
       </c>
       <c r="H1309" s="3"/>
       <c r="I1309" s="3"/>
@@ -53637,7 +53898,7 @@
     </row>
     <row r="1310" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1310" s="3" t="s">
-        <v>3684</v>
+        <v>3683</v>
       </c>
       <c r="B1310" s="3" t="s">
         <v>62</v>
@@ -53652,10 +53913,10 @@
         <v>80</v>
       </c>
       <c r="F1310" s="3" t="s">
+        <v>3684</v>
+      </c>
+      <c r="G1310" s="3" t="s">
         <v>3685</v>
-      </c>
-      <c r="G1310" s="3" t="s">
-        <v>3686</v>
       </c>
       <c r="H1310" s="3" t="s">
         <v>37</v>
@@ -53669,15 +53930,15 @@
         <v>39</v>
       </c>
       <c r="M1310" s="3" t="s">
+        <v>3686</v>
+      </c>
+      <c r="N1310" s="3" t="s">
         <v>3687</v>
-      </c>
-      <c r="N1310" s="3" t="s">
-        <v>3688</v>
       </c>
     </row>
     <row r="1311" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1311" s="3" t="s">
-        <v>3689</v>
+        <v>3688</v>
       </c>
       <c r="B1311" s="3"/>
       <c r="C1311" s="3">
@@ -53690,10 +53951,10 @@
         <v>80</v>
       </c>
       <c r="F1311" s="3" t="s">
+        <v>3689</v>
+      </c>
+      <c r="G1311" s="3" t="s">
         <v>3690</v>
-      </c>
-      <c r="G1311" s="3" t="s">
-        <v>3691</v>
       </c>
       <c r="H1311" s="3"/>
       <c r="I1311" s="3"/>
@@ -53705,15 +53966,17 @@
         <v>39</v>
       </c>
       <c r="M1311" s="3" t="s">
-        <v>3692</v>
+        <v>3691</v>
       </c>
       <c r="N1311" s="3"/>
     </row>
     <row r="1312" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1312" s="3" t="s">
-        <v>3693</v>
-      </c>
-      <c r="B1312" s="3"/>
+        <v>3692</v>
+      </c>
+      <c r="B1312" s="3" t="s">
+        <v>3456</v>
+      </c>
       <c r="C1312" s="3">
         <v>111</v>
       </c>
@@ -53724,13 +53987,13 @@
         <v>80</v>
       </c>
       <c r="F1312" s="3" t="s">
+        <v>3693</v>
+      </c>
+      <c r="G1312" s="3" t="s">
         <v>3694</v>
       </c>
-      <c r="G1312" s="3" t="s">
-        <v>3695</v>
-      </c>
       <c r="H1312" s="3" t="s">
-        <v>1678</v>
+        <v>37</v>
       </c>
       <c r="I1312" s="3"/>
       <c r="J1312" s="3"/>
@@ -53741,9 +54004,11 @@
         <v>39</v>
       </c>
       <c r="M1312" s="3" t="s">
+        <v>3695</v>
+      </c>
+      <c r="N1312" s="3" t="s">
         <v>3696</v>
       </c>
-      <c r="N1312" s="3"/>
     </row>
     <row r="1313" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1313" s="3" t="s">
@@ -53895,6 +54160,898 @@
       <c r="M1317" s="3"/>
       <c r="N1317" s="3"/>
     </row>
+    <row r="1318" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1318" s="3" t="s">
+        <v>3712</v>
+      </c>
+      <c r="B1318" s="3"/>
+      <c r="C1318" s="3">
+        <v>112</v>
+      </c>
+      <c r="D1318" s="3">
+        <v>6252427157</v>
+      </c>
+      <c r="E1318" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1318" s="3" t="s">
+        <v>3713</v>
+      </c>
+      <c r="G1318" s="3" t="s">
+        <v>3714</v>
+      </c>
+      <c r="H1318" s="3"/>
+      <c r="I1318" s="3"/>
+      <c r="J1318" s="3"/>
+      <c r="K1318" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1318" s="3"/>
+      <c r="M1318" s="3"/>
+      <c r="N1318" s="3"/>
+    </row>
+    <row r="1319" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1319" s="3" t="s">
+        <v>3715</v>
+      </c>
+      <c r="B1319" s="3"/>
+      <c r="C1319" s="3">
+        <v>111</v>
+      </c>
+      <c r="D1319" s="3">
+        <v>6252909778</v>
+      </c>
+      <c r="E1319" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1319" s="3" t="s">
+        <v>1710</v>
+      </c>
+      <c r="G1319" s="3" t="s">
+        <v>3716</v>
+      </c>
+      <c r="H1319" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I1319" s="3"/>
+      <c r="J1319" s="3"/>
+      <c r="K1319" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1319" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1319" s="3" t="s">
+        <v>3717</v>
+      </c>
+      <c r="N1319" s="3"/>
+    </row>
+    <row r="1320" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1320" s="3" t="s">
+        <v>3718</v>
+      </c>
+      <c r="B1320" s="3"/>
+      <c r="C1320" s="3">
+        <v>112</v>
+      </c>
+      <c r="D1320" s="3">
+        <v>6263491722</v>
+      </c>
+      <c r="E1320" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1320" s="3" t="s">
+        <v>3719</v>
+      </c>
+      <c r="G1320" s="3" t="s">
+        <v>3720</v>
+      </c>
+      <c r="H1320" s="3"/>
+      <c r="I1320" s="3"/>
+      <c r="J1320" s="3"/>
+      <c r="K1320" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1320" s="3"/>
+      <c r="M1320" s="3"/>
+      <c r="N1320" s="3"/>
+    </row>
+    <row r="1321" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1321" s="3" t="s">
+        <v>3721</v>
+      </c>
+      <c r="B1321" s="3"/>
+      <c r="C1321" s="3">
+        <v>113</v>
+      </c>
+      <c r="D1321" s="3">
+        <v>6263775709</v>
+      </c>
+      <c r="E1321" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1321" s="3" t="s">
+        <v>2146</v>
+      </c>
+      <c r="G1321" s="3" t="s">
+        <v>3722</v>
+      </c>
+      <c r="H1321" s="3"/>
+      <c r="I1321" s="3"/>
+      <c r="J1321" s="3"/>
+      <c r="K1321" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1321" s="3"/>
+      <c r="M1321" s="3"/>
+      <c r="N1321" s="3"/>
+    </row>
+    <row r="1322" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1322" s="3" t="s">
+        <v>3723</v>
+      </c>
+      <c r="B1322" s="3"/>
+      <c r="C1322" s="3">
+        <v>112</v>
+      </c>
+      <c r="D1322" s="3">
+        <v>6259132121</v>
+      </c>
+      <c r="E1322" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1322" s="3" t="s">
+        <v>3724</v>
+      </c>
+      <c r="G1322" s="3" t="s">
+        <v>3725</v>
+      </c>
+      <c r="H1322" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I1322" s="3"/>
+      <c r="J1322" s="3"/>
+      <c r="K1322" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1322" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1322" s="3" t="s">
+        <v>3650</v>
+      </c>
+      <c r="N1322" s="3"/>
+    </row>
+    <row r="1323" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1323" s="3" t="s">
+        <v>3726</v>
+      </c>
+      <c r="B1323" s="3"/>
+      <c r="C1323" s="3">
+        <v>112</v>
+      </c>
+      <c r="D1323" s="3">
+        <v>6259362876</v>
+      </c>
+      <c r="E1323" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1323" s="3" t="s">
+        <v>3727</v>
+      </c>
+      <c r="G1323" s="3" t="s">
+        <v>3728</v>
+      </c>
+      <c r="H1323" s="3"/>
+      <c r="I1323" s="3"/>
+      <c r="J1323" s="3"/>
+      <c r="K1323" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1323" s="3"/>
+      <c r="M1323" s="3"/>
+      <c r="N1323" s="3"/>
+    </row>
+    <row r="1324" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1324" s="3" t="s">
+        <v>3729</v>
+      </c>
+      <c r="B1324" s="3"/>
+      <c r="C1324" s="3">
+        <v>112</v>
+      </c>
+      <c r="D1324" s="3">
+        <v>6270898497</v>
+      </c>
+      <c r="E1324" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1324" s="3" t="s">
+        <v>3730</v>
+      </c>
+      <c r="G1324" s="3" t="s">
+        <v>3731</v>
+      </c>
+      <c r="H1324" s="3"/>
+      <c r="I1324" s="3"/>
+      <c r="J1324" s="3"/>
+      <c r="K1324" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1324" s="3"/>
+      <c r="M1324" s="3"/>
+      <c r="N1324" s="3"/>
+    </row>
+    <row r="1325" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1325" s="3" t="s">
+        <v>3732</v>
+      </c>
+      <c r="B1325" s="3"/>
+      <c r="C1325" s="3">
+        <v>112</v>
+      </c>
+      <c r="D1325" s="3">
+        <v>6260883890</v>
+      </c>
+      <c r="E1325" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1325" s="3" t="s">
+        <v>3733</v>
+      </c>
+      <c r="G1325" s="3" t="s">
+        <v>3734</v>
+      </c>
+      <c r="H1325" s="3"/>
+      <c r="I1325" s="3"/>
+      <c r="J1325" s="3"/>
+      <c r="K1325" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1325" s="3"/>
+      <c r="M1325" s="3"/>
+      <c r="N1325" s="3"/>
+    </row>
+    <row r="1326" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1326" s="3" t="s">
+        <v>3735</v>
+      </c>
+      <c r="B1326" s="3"/>
+      <c r="C1326" s="3">
+        <v>112</v>
+      </c>
+      <c r="D1326" s="3">
+        <v>6260934691</v>
+      </c>
+      <c r="E1326" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1326" s="3" t="s">
+        <v>3736</v>
+      </c>
+      <c r="G1326" s="3" t="s">
+        <v>3737</v>
+      </c>
+      <c r="H1326" s="3"/>
+      <c r="I1326" s="3"/>
+      <c r="J1326" s="3"/>
+      <c r="K1326" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1326" s="3"/>
+      <c r="M1326" s="3"/>
+      <c r="N1326" s="3"/>
+    </row>
+    <row r="1327" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1327" s="3" t="s">
+        <v>3738</v>
+      </c>
+      <c r="B1327" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1327" s="3">
+        <v>301</v>
+      </c>
+      <c r="D1327" s="3">
+        <v>6265025587</v>
+      </c>
+      <c r="E1327" s="3" t="s">
+        <v>2371</v>
+      </c>
+      <c r="F1327" s="3" t="s">
+        <v>3739</v>
+      </c>
+      <c r="G1327" s="3" t="s">
+        <v>3740</v>
+      </c>
+      <c r="H1327" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I1327" s="3"/>
+      <c r="J1327" s="3"/>
+      <c r="K1327" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1327" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1327" s="3" t="s">
+        <v>3741</v>
+      </c>
+      <c r="N1327" s="3"/>
+    </row>
+    <row r="1328" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1328" s="3" t="s">
+        <v>3742</v>
+      </c>
+      <c r="B1328" s="3"/>
+      <c r="C1328" s="3">
+        <v>113</v>
+      </c>
+      <c r="D1328" s="3">
+        <v>6265080307</v>
+      </c>
+      <c r="E1328" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="F1328" s="3" t="s">
+        <v>3743</v>
+      </c>
+      <c r="G1328" s="3" t="s">
+        <v>3744</v>
+      </c>
+      <c r="H1328" s="3"/>
+      <c r="I1328" s="3"/>
+      <c r="J1328" s="3"/>
+      <c r="K1328" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1328" s="3"/>
+      <c r="M1328" s="3"/>
+      <c r="N1328" s="3"/>
+    </row>
+    <row r="1329" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1329" s="3" t="s">
+        <v>3745</v>
+      </c>
+      <c r="B1329" s="3"/>
+      <c r="C1329" s="3">
+        <v>301</v>
+      </c>
+      <c r="D1329" s="3">
+        <v>6265580906</v>
+      </c>
+      <c r="E1329" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="F1329" s="3" t="s">
+        <v>2258</v>
+      </c>
+      <c r="G1329" s="3" t="s">
+        <v>3746</v>
+      </c>
+      <c r="H1329" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I1329" s="3"/>
+      <c r="J1329" s="3"/>
+      <c r="K1329" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1329" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1329" s="3" t="s">
+        <v>3747</v>
+      </c>
+      <c r="N1329" s="3"/>
+    </row>
+    <row r="1330" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1330" s="3" t="s">
+        <v>3748</v>
+      </c>
+      <c r="B1330" s="3"/>
+      <c r="C1330" s="3">
+        <v>113</v>
+      </c>
+      <c r="D1330" s="3">
+        <v>6266882286</v>
+      </c>
+      <c r="E1330" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1330" s="3" t="s">
+        <v>3749</v>
+      </c>
+      <c r="G1330" s="3" t="s">
+        <v>3750</v>
+      </c>
+      <c r="H1330" s="3"/>
+      <c r="I1330" s="3"/>
+      <c r="J1330" s="3"/>
+      <c r="K1330" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1330" s="3"/>
+      <c r="M1330" s="3"/>
+      <c r="N1330" s="3"/>
+    </row>
+    <row r="1331" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1331" s="3" t="s">
+        <v>3751</v>
+      </c>
+      <c r="B1331" s="3"/>
+      <c r="C1331" s="3">
+        <v>113</v>
+      </c>
+      <c r="D1331" s="3">
+        <v>6277977155</v>
+      </c>
+      <c r="E1331" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1331" s="3" t="s">
+        <v>3752</v>
+      </c>
+      <c r="G1331" s="3" t="s">
+        <v>3753</v>
+      </c>
+      <c r="H1331" s="3"/>
+      <c r="I1331" s="3"/>
+      <c r="J1331" s="3"/>
+      <c r="K1331" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1331" s="3"/>
+      <c r="M1331" s="3"/>
+      <c r="N1331" s="3"/>
+    </row>
+    <row r="1332" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1332" s="3" t="s">
+        <v>3754</v>
+      </c>
+      <c r="B1332" s="3"/>
+      <c r="C1332" s="3">
+        <v>113</v>
+      </c>
+      <c r="D1332" s="3">
+        <v>6269974762</v>
+      </c>
+      <c r="E1332" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1332" s="3" t="s">
+        <v>3755</v>
+      </c>
+      <c r="G1332" s="3" t="s">
+        <v>3756</v>
+      </c>
+      <c r="H1332" s="3"/>
+      <c r="I1332" s="3"/>
+      <c r="J1332" s="3"/>
+      <c r="K1332" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1332" s="3"/>
+      <c r="M1332" s="3"/>
+      <c r="N1332" s="3"/>
+    </row>
+    <row r="1333" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1333" s="3" t="s">
+        <v>3757</v>
+      </c>
+      <c r="B1333" s="3"/>
+      <c r="C1333" s="3">
+        <v>113</v>
+      </c>
+      <c r="D1333" s="3">
+        <v>6272071925</v>
+      </c>
+      <c r="E1333" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1333" s="3" t="s">
+        <v>3758</v>
+      </c>
+      <c r="G1333" s="3" t="s">
+        <v>3759</v>
+      </c>
+      <c r="H1333" s="3"/>
+      <c r="I1333" s="3"/>
+      <c r="J1333" s="3"/>
+      <c r="K1333" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1333" s="3"/>
+      <c r="M1333" s="3"/>
+      <c r="N1333" s="3"/>
+    </row>
+    <row r="1334" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1334" s="3" t="s">
+        <v>3760</v>
+      </c>
+      <c r="B1334" s="3"/>
+      <c r="C1334" s="3">
+        <v>113</v>
+      </c>
+      <c r="D1334" s="3">
+        <v>6273858561</v>
+      </c>
+      <c r="E1334" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1334" s="3" t="s">
+        <v>3761</v>
+      </c>
+      <c r="G1334" s="3" t="s">
+        <v>3762</v>
+      </c>
+      <c r="H1334" s="3"/>
+      <c r="I1334" s="3"/>
+      <c r="J1334" s="3"/>
+      <c r="K1334" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1334" s="3"/>
+      <c r="M1334" s="3"/>
+      <c r="N1334" s="3"/>
+    </row>
+    <row r="1335" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1335" s="3" t="s">
+        <v>3763</v>
+      </c>
+      <c r="B1335" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1335" s="3">
+        <v>110</v>
+      </c>
+      <c r="D1335" s="3">
+        <v>6274453367</v>
+      </c>
+      <c r="E1335" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1335" s="3" t="s">
+        <v>3764</v>
+      </c>
+      <c r="G1335" s="3" t="s">
+        <v>3765</v>
+      </c>
+      <c r="H1335" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I1335" s="3"/>
+      <c r="J1335" s="3"/>
+      <c r="K1335" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1335" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1335" s="3" t="s">
+        <v>3766</v>
+      </c>
+      <c r="N1335" s="3"/>
+    </row>
+    <row r="1336" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1336" s="3" t="s">
+        <v>3767</v>
+      </c>
+      <c r="B1336" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1336" s="3">
+        <v>110</v>
+      </c>
+      <c r="D1336" s="3">
+        <v>6274525700</v>
+      </c>
+      <c r="E1336" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1336" s="3" t="s">
+        <v>3768</v>
+      </c>
+      <c r="G1336" s="3" t="s">
+        <v>3769</v>
+      </c>
+      <c r="H1336" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I1336" s="3"/>
+      <c r="J1336" s="3"/>
+      <c r="K1336" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1336" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1336" s="3" t="s">
+        <v>3770</v>
+      </c>
+      <c r="N1336" s="3"/>
+    </row>
+    <row r="1337" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1337" s="3" t="s">
+        <v>3771</v>
+      </c>
+      <c r="B1337" s="3"/>
+      <c r="C1337" s="3">
+        <v>112</v>
+      </c>
+      <c r="D1337" s="3">
+        <v>6284567772</v>
+      </c>
+      <c r="E1337" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1337" s="3" t="s">
+        <v>3772</v>
+      </c>
+      <c r="G1337" s="3" t="s">
+        <v>3773</v>
+      </c>
+      <c r="H1337" s="3"/>
+      <c r="I1337" s="3"/>
+      <c r="J1337" s="3"/>
+      <c r="K1337" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1337" s="3"/>
+      <c r="M1337" s="3"/>
+      <c r="N1337" s="3"/>
+    </row>
+    <row r="1338" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1338" s="3" t="s">
+        <v>3774</v>
+      </c>
+      <c r="B1338" s="3"/>
+      <c r="C1338" s="3">
+        <v>111</v>
+      </c>
+      <c r="D1338" s="3">
+        <v>6277432874</v>
+      </c>
+      <c r="E1338" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1338" s="3" t="s">
+        <v>3775</v>
+      </c>
+      <c r="G1338" s="3" t="s">
+        <v>3776</v>
+      </c>
+      <c r="H1338" s="3"/>
+      <c r="I1338" s="3"/>
+      <c r="J1338" s="3"/>
+      <c r="K1338" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1338" s="3"/>
+      <c r="M1338" s="3"/>
+      <c r="N1338" s="3"/>
+    </row>
+    <row r="1339" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1339" s="3" t="s">
+        <v>3777</v>
+      </c>
+      <c r="B1339" s="3"/>
+      <c r="C1339" s="3">
+        <v>111</v>
+      </c>
+      <c r="D1339" s="3">
+        <v>6277442024</v>
+      </c>
+      <c r="E1339" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1339" s="3" t="s">
+        <v>3778</v>
+      </c>
+      <c r="G1339" s="3" t="s">
+        <v>3779</v>
+      </c>
+      <c r="H1339" s="3"/>
+      <c r="I1339" s="3"/>
+      <c r="J1339" s="3"/>
+      <c r="K1339" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1339" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1339" s="3" t="s">
+        <v>3780</v>
+      </c>
+      <c r="N1339" s="3"/>
+    </row>
+    <row r="1340" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1340" s="3" t="s">
+        <v>3781</v>
+      </c>
+      <c r="B1340" s="3"/>
+      <c r="C1340" s="3">
+        <v>112</v>
+      </c>
+      <c r="D1340" s="3">
+        <v>6279742775</v>
+      </c>
+      <c r="E1340" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="F1340" s="3" t="s">
+        <v>3782</v>
+      </c>
+      <c r="G1340" s="3" t="s">
+        <v>3783</v>
+      </c>
+      <c r="H1340" s="3"/>
+      <c r="I1340" s="3"/>
+      <c r="J1340" s="3"/>
+      <c r="K1340" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1340" s="3"/>
+      <c r="M1340" s="3"/>
+      <c r="N1340" s="3"/>
+    </row>
+    <row r="1341" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1341" s="3" t="s">
+        <v>3784</v>
+      </c>
+      <c r="B1341" s="3"/>
+      <c r="C1341" s="3">
+        <v>113</v>
+      </c>
+      <c r="D1341" s="3">
+        <v>6289278890</v>
+      </c>
+      <c r="E1341" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1341" s="3" t="s">
+        <v>3785</v>
+      </c>
+      <c r="G1341" s="3" t="s">
+        <v>3786</v>
+      </c>
+      <c r="H1341" s="3"/>
+      <c r="I1341" s="3"/>
+      <c r="J1341" s="3"/>
+      <c r="K1341" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1341" s="3"/>
+      <c r="M1341" s="3"/>
+      <c r="N1341" s="3"/>
+    </row>
+    <row r="1342" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1342" s="3" t="s">
+        <v>3787</v>
+      </c>
+      <c r="B1342" s="3"/>
+      <c r="C1342" s="3">
+        <v>113</v>
+      </c>
+      <c r="D1342" s="3">
+        <v>6289116067</v>
+      </c>
+      <c r="E1342" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1342" s="3" t="s">
+        <v>3788</v>
+      </c>
+      <c r="G1342" s="3" t="s">
+        <v>3789</v>
+      </c>
+      <c r="H1342" s="3"/>
+      <c r="I1342" s="3"/>
+      <c r="J1342" s="3"/>
+      <c r="K1342" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1342" s="3"/>
+      <c r="M1342" s="3"/>
+      <c r="N1342" s="3"/>
+    </row>
+    <row r="1343" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1343" s="3" t="s">
+        <v>3790</v>
+      </c>
+      <c r="B1343" s="3"/>
+      <c r="C1343" s="3">
+        <v>112</v>
+      </c>
+      <c r="D1343" s="3">
+        <v>6282853132</v>
+      </c>
+      <c r="E1343" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1343" s="3" t="s">
+        <v>1333</v>
+      </c>
+      <c r="G1343" s="3" t="s">
+        <v>3791</v>
+      </c>
+      <c r="H1343" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I1343" s="3"/>
+      <c r="J1343" s="3"/>
+      <c r="K1343" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1343" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1343" s="3" t="s">
+        <v>3792</v>
+      </c>
+      <c r="N1343" s="3"/>
+    </row>
+    <row r="1344" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1344" s="3" t="s">
+        <v>3793</v>
+      </c>
+      <c r="B1344" s="3"/>
+      <c r="C1344" s="3">
+        <v>111</v>
+      </c>
+      <c r="D1344" s="3">
+        <v>6285690638</v>
+      </c>
+      <c r="E1344" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1344" s="3" t="s">
+        <v>3794</v>
+      </c>
+      <c r="G1344" s="3" t="s">
+        <v>3795</v>
+      </c>
+      <c r="H1344" s="3"/>
+      <c r="I1344" s="3"/>
+      <c r="J1344" s="3"/>
+      <c r="K1344" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1344" s="3"/>
+      <c r="M1344" s="3"/>
+      <c r="N1344" s="3"/>
+    </row>
+    <row r="1345" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1345" s="3" t="s">
+        <v>3796</v>
+      </c>
+      <c r="B1345" s="3"/>
+      <c r="C1345" s="3">
+        <v>111</v>
+      </c>
+      <c r="D1345" s="3">
+        <v>6286015689</v>
+      </c>
+      <c r="E1345" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1345" s="3" t="s">
+        <v>3797</v>
+      </c>
+      <c r="G1345" s="3" t="s">
+        <v>3798</v>
+      </c>
+      <c r="H1345" s="3"/>
+      <c r="I1345" s="3"/>
+      <c r="J1345" s="3"/>
+      <c r="K1345" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1345" s="3"/>
+      <c r="M1345" s="3"/>
+      <c r="N1345" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>